<commit_message>
Ajout nouvelle ligne Feuille DEV
</commit_message>
<xml_diff>
--- a/Base_Connaissances_Excel/Feuille de calcul de la base de connaissance-1.xlsx
+++ b/Base_Connaissances_Excel/Feuille de calcul de la base de connaissance-1.xlsx
@@ -5,16 +5,16 @@
   <workbookPr showInkAnnotation="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\latitude\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\latitude\Desktop\Projets-fil-rouge\Base_Connaissances_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD628A2A-B836-45B2-960B-EDB50E325096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E536E4-D6CB-4D91-BC36-F12699A85FC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Entrées base de connaissances " sheetId="3" r:id="rId1"/>
-    <sheet name="Entrées base de connaissanc (2)" sheetId="10" r:id="rId2"/>
+    <sheet name="Entrées BC AWS Cloud" sheetId="3" r:id="rId1"/>
+    <sheet name="Entrées BC WEB" sheetId="10" r:id="rId2"/>
     <sheet name="Entrées base de connaissanc (3)" sheetId="11" r:id="rId3"/>
     <sheet name="catégories" sheetId="9" r:id="rId4"/>
   </sheets>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="71">
   <si>
     <t>Commentaires</t>
   </si>
@@ -401,12 +401,80 @@
   <si>
     <t>178--Lab - Utilisation d'AWS Lambda</t>
   </si>
+  <si>
+    <t>Git</t>
+  </si>
+  <si>
+    <t>Problème de gestion Git dû à un projet local mal organisé (plusieurs dossiers et fichiers untracked) qui a provoqué des conflits entre branches, le blocage des changements de branche et des push contenant des fichiers non désirés.</t>
+  </si>
+  <si>
+    <t>Impossible de changer de branche à cause de fichiers “untracked” bloquants, push contenant des fichiers inattendus, et apparition de dossiers non souhaités dans le staging ou les commits.</t>
+  </si>
+  <si>
+    <t>La cause racine est un dépôt local mal structuré où plusieurs projets et dépendances (V1, V2, node_modules) coexistaient sans séparation ni .gitignore correct, combiné à une mauvaise isolation des branches, ce qui a fait que Git a mélangé fichiers locaux non suivis et historique de commits entre branches.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Créer une branche totalement propre (sans historique):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="22"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Amazon Ember Light"/>
+      </rPr>
+      <t>git checkout --orphan nouvelle-branche</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="22"/>
+        <color theme="1"/>
+        <rFont val="Amazon Ember Light"/>
+      </rPr>
+      <t xml:space="preserve">
+Supprimer tous les fichiers suivis du staging:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="22"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Amazon Ember Light"/>
+      </rPr>
+      <t>git rm -rf .</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="22"/>
+        <color theme="1"/>
+        <rFont val="Amazon Ember Light"/>
+      </rPr>
+      <t xml:space="preserve">
+Ajouter uniquement le dossier qu'on veut ajouter
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="22"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Amazon Ember Light"/>
+      </rPr>
+      <t>git add ton_dossier/</t>
+    </r>
+  </si>
+  <si>
+    <t>Documentation GIT</t>
+  </si>
+  <si>
+    <t>Se reférer à la documentation pour resoudre se genre de problème</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -477,6 +545,11 @@
     <font>
       <sz val="22"/>
       <color rgb="FF000000"/>
+      <name val="Amazon Ember Light"/>
+    </font>
+    <font>
+      <sz val="22"/>
+      <color rgb="FFFF0000"/>
       <name val="Amazon Ember Light"/>
     </font>
   </fonts>
@@ -1839,116 +1912,41 @@
         <v>15</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>14</v>
+        <v>64</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>12</v>
+        <v>66</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="I2" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="279.89999999999998" customHeight="1">
-      <c r="A3" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="I3" s="17" t="s">
-        <v>16</v>
-      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:9" ht="207" customHeight="1">
-      <c r="A4" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="I4" s="17" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="207" customHeight="1" thickBot="1">
-      <c r="A5" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="F5" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5" s="22" t="s">
-        <v>30</v>
-      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" ht="207" customHeight="1">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:9" ht="22.8">
       <c r="A6" s="5"/>
@@ -3272,21 +3270,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010006807B066C556C4DA1F97EE96CC1104B" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="cfb987611df5cdae7f7a5067c3395bc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c2ee6f6c-285d-4b95-ace0-9682ebe56039" xmlns:ns3="012b183d-1ada-4ff6-b855-98c4d59bda2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08f2586826dc5d0b05e832f2b79fc23a" ns2:_="" ns3:_="">
     <xsd:import namespace="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
@@ -3509,10 +3492,36 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
+    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3535,20 +3544,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
-    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>